<commit_message>
Q2 2026 data processing + script updates
Converted scripts to typescript and improved error reporting
Fixed issues with wqx delete file creation
Added script for importing wqx data from EPA WQP
Support for Lanai in wqx and aqualink data processing
</commit_message>
<xml_diff>
--- a/reports/web-export-quarterly-reports/web-export-starting-file-South-Maui.xlsx
+++ b/reports/web-export-quarterly-reports/web-export-starting-file-South-Maui.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10509"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10802"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bill/development/water-quality/hui-reports/reports/web-export-quarterly-reports/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dan/hui/hui-reports/reports/web-export-quarterly-reports/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F22983F-4F16-1C4B-83AD-BAE2CAA65411}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6128BF2-FC9E-BA41-A4F7-3EBC75468B50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20060" yWindow="2700" windowWidth="32160" windowHeight="22420" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="meta data" sheetId="2" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="130407" concurrentCalc="0"/>
+  <calcPr calcId="130407"/>
   <extLst>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{7523E5D3-25F3-A5E0-1632-64F254C22452}">
       <mx:ArchID Flags="2"/>
@@ -154,9 +154,6 @@
     <t>Time</t>
   </si>
   <si>
-    <t>Falinski, Kim, Reed, Dana, Callender, Tova, Fielding, Emily, Newbold, Robin, &amp; Yurkanin, Alana. (2017). Hui o ka Wai Ola Water Quality Data [Data set]. Zenodo. http://doi.org/10.5281/zenodo.830049</t>
-  </si>
-  <si>
     <t>APHA Method 4500-P, GF/F-filtered grab samples, SEAL Analytical AA3 autoanalyzer</t>
   </si>
   <si>
@@ -197,6 +194,9 @@
   </si>
   <si>
     <t>Ammonium-OPA Method, GF/F-filtered grab samples, SEAL Analytical AA3 autoanalyzer</t>
+  </si>
+  <si>
+    <t>Hui O Ka Wai Ola Water Quality Data. https://www.huiokawaiola.com/data.html</t>
   </si>
 </sst>
 </file>
@@ -248,7 +248,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -260,9 +260,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -641,12 +638,12 @@
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
     </row>
-    <row r="4" spans="1:4" ht="64" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" ht="32" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>15</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
@@ -669,20 +666,20 @@
     </row>
     <row r="7" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
     </row>
     <row r="8" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>50</v>
       </c>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
@@ -692,17 +689,17 @@
         <v>39</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
     </row>
     <row r="10" spans="1:4" ht="32" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
@@ -822,7 +819,7 @@
         <v>33</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="32" x14ac:dyDescent="0.2">
@@ -836,7 +833,7 @@
         <v>33</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="32" x14ac:dyDescent="0.2">
@@ -850,7 +847,7 @@
         <v>33</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="32" x14ac:dyDescent="0.2">
@@ -864,7 +861,7 @@
         <v>33</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="32" x14ac:dyDescent="0.2">
@@ -878,7 +875,7 @@
         <v>33</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="34" customHeight="1" x14ac:dyDescent="0.2">
@@ -886,13 +883,13 @@
         <v>11</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>33</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="15" x14ac:dyDescent="0.2">
@@ -903,7 +900,7 @@
     </row>
     <row r="26" spans="1:4" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="1"/>
-      <c r="B26" s="5" t="s">
+      <c r="B26" s="4" t="s">
         <v>38</v>
       </c>
       <c r="C26" s="4"/>
@@ -911,9 +908,9 @@
     </row>
     <row r="27" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A27" s="1"/>
-      <c r="B27" s="6"/>
-      <c r="C27" s="6"/>
-      <c r="D27" s="6"/>
+      <c r="B27" s="5"/>
+      <c r="C27" s="5"/>
+      <c r="D27" s="5"/>
     </row>
     <row r="28" spans="1:4" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="e">

</xml_diff>